<commit_message>
Organize each control into CDA and CPA folders with Reference Folders Reviewed blocks
Testing Procedures split into CDA (questions 1-10) and CPA (sampling and test steps) documents; process map and population under CDA, sample evidence under CPA\S1 Security Lending and CPA\S2 NDF; evidence named BSI.IT.23.Cx.nn - description; every reference block rewritten to name the folder and files; index and packages updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkbhuE8rWvfJG8fUAag8f1
</commit_message>
<xml_diff>
--- a/SDLC2026 BSI/00 Summary and Evidence Index.xlsx
+++ b/SDLC2026 BSI/00 Summary and Evidence Index.xlsx
@@ -538,7 +538,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -614,12 +613,12 @@
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Testing Procedures / Audit Workpapers</t>
+          <t>Folder structure</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Each control folder holds a Testing Procedures document (Cx Testing Procedures.docx) (C25 format, no tables) and an IT Audit Workpaper – Sample Size of 1 (Cx Audit Workpaper.docx) answering every test step for each of the two samples with inline evidence references.</t>
+          <t>Each control folder holds the workbook (Cx WP 2026.xlsm) and two sub-folders. CDA: Cx Control Design Assessment - CDA.docx (questions 1 – 10), Cx Design Walkthrough Sample of 1.docx and the folder "Process Map and Population". CPA: Cx Control Performance Assessment - CPA.docx (sampling and test steps), Cx Audit Workpaper (Sample Size 1).docx and the sample folders "S1 Security Lending" and "S2 NDF". Every answer ends with "Reference Folders Reviewed" naming the folder and files.</t>
         </is>
       </c>
     </row>
@@ -935,7 +934,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
@@ -1254,7 +1252,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -1288,7 +1285,7 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>File in work folder (link)</t>
+          <t>File in work folder (link) – CDA = process map &amp; population, CPA = sample evidence</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
@@ -1330,7 +1327,7 @@
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/00 Common/C1.01 - 2026 SDLC process map.pdf</t>
+          <t>C1 Business Req/CDA/Process Map and Population/BSI.IT.23.C1.01 - 2026 SDLC Process Map.pdf</t>
         </is>
       </c>
       <c r="H5" s="12" t="inlineStr">
@@ -1372,7 +1369,7 @@
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/00 Common/C1.02 - SDLC Project List.xlsx</t>
+          <t>C1 Business Req/CDA/Process Map and Population/BSI.IT.23.C1.02 - SDLC Project List (population).xlsx</t>
         </is>
       </c>
       <c r="H6" s="12" t="inlineStr">
@@ -1414,7 +1411,7 @@
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/S1 SecLending/C1.03 - SL R01 BRD.docx</t>
+          <t>C1 Business Req/CPA/S1 Security Lending/BSI.IT.23.C1.03 - Security Lending R01 BRD.docx</t>
         </is>
       </c>
       <c r="H7" s="12" t="inlineStr">
@@ -1456,7 +1453,7 @@
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/S1 SecLending/C1.04 - SL R01 sponsor approval 02-06-2026.msg</t>
+          <t>C1 Business Req/CPA/S1 Security Lending/BSI.IT.23.C1.04 - Security Lending R01 sponsor approval 02-06-2026.msg</t>
         </is>
       </c>
       <c r="H8" s="12" t="inlineStr">
@@ -1498,7 +1495,7 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/S1 SecLending/C1.05 - SL R02 BRD.docx</t>
+          <t>C1 Business Req/CPA/S1 Security Lending/BSI.IT.23.C1.05 - Security Lending R02 BRD.docx</t>
         </is>
       </c>
       <c r="H9" s="12" t="inlineStr">
@@ -1540,7 +1537,7 @@
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/S1 SecLending/C1.06 - SL R02 sponsor approval 04-29-2026.msg</t>
+          <t>C1 Business Req/CPA/S1 Security Lending/BSI.IT.23.C1.06 - Security Lending R02 sponsor approval 04-29-2026.msg</t>
         </is>
       </c>
       <c r="H10" s="12" t="inlineStr">
@@ -1582,7 +1579,7 @@
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/S2 NDF/C1.07 - NDF R01 BRD.docx</t>
+          <t>C1 Business Req/CPA/S2 NDF/BSI.IT.23.C1.07 - NDF R01 BRD.docx</t>
         </is>
       </c>
       <c r="H11" s="12" t="inlineStr">
@@ -1624,7 +1621,7 @@
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/S2 NDF/C1.08 - NDF R01 sponsor sign-off 10-23-2025.msg</t>
+          <t>C1 Business Req/CPA/S2 NDF/BSI.IT.23.C1.08 - NDF R01 sponsor sign-off 10-23-2025.msg</t>
         </is>
       </c>
       <c r="H12" s="12" t="inlineStr">
@@ -1666,7 +1663,7 @@
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/S2 NDF/C1.09 - NDF R01 Gate 4 11-04-2025.pdf</t>
+          <t>C1 Business Req/CPA/S2 NDF/BSI.IT.23.C1.09 - NDF R01 Gate 4 approval 11-04-2025.pdf</t>
         </is>
       </c>
       <c r="H13" s="12" t="inlineStr">
@@ -1708,7 +1705,7 @@
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/S2 NDF/C1.10 - NDF R02 BRD.docx</t>
+          <t>C1 Business Req/CPA/S2 NDF/BSI.IT.23.C1.10 - NDF R02 BRD.docx</t>
         </is>
       </c>
       <c r="H14" s="12" t="inlineStr">
@@ -1750,7 +1747,7 @@
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/S2 NDF/C1.11 - NDF R02 sponsor sign-off 12-02-2025.msg</t>
+          <t>C1 Business Req/CPA/S2 NDF/BSI.IT.23.C1.11 - NDF R02 sponsor sign-off 12-02-2025.msg</t>
         </is>
       </c>
       <c r="H15" s="12" t="inlineStr">
@@ -1792,7 +1789,7 @@
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/S2 NDF/C1.12 - NDF R02 Gate 4 03-10-2026.pdf</t>
+          <t>C1 Business Req/CPA/S2 NDF/BSI.IT.23.C1.12 - NDF R02 Gate 4 approval 03-10-2026.pdf</t>
         </is>
       </c>
       <c r="H16" s="12" t="inlineStr">
@@ -1834,7 +1831,7 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/S1 SecLending/C1.13 - SL gate dispositions.docx</t>
+          <t>C1 Business Req/CPA/S1 Security Lending/BSI.IT.23.C1.13 - Security Lending gate history (PTB 10-31-2025).docx</t>
         </is>
       </c>
       <c r="H17" s="12" t="inlineStr">
@@ -1876,7 +1873,7 @@
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/S1 SecLending/C1.14 - SL Appian release emails 02-2026.msg</t>
+          <t>C1 Business Req/CPA/S1 Security Lending/BSI.IT.23.C1.14 - Security Lending Appian release emails 02-2026.msg</t>
         </is>
       </c>
       <c r="H18" s="12" t="inlineStr">
@@ -1918,7 +1915,7 @@
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>C1 Business Req/Evidence/S1 SecLending/C1.15 - SL T24 release emails 05-2026.msg</t>
+          <t>C1 Business Req/CPA/S1 Security Lending/BSI.IT.23.C1.15 - Security Lending T24 release emails 05-2026.msg</t>
         </is>
       </c>
       <c r="H19" s="12" t="inlineStr">
@@ -1960,7 +1957,7 @@
       </c>
       <c r="G20" s="13" t="inlineStr">
         <is>
-          <t>C13 Design of System/Evidence/00 Common/C13.01 - 2026 SDLC process map.pdf</t>
+          <t>C13 Design of System/CDA/Process Map and Population/BSI.IT.23.C13.01 - 2026 SDLC Process Map.pdf</t>
         </is>
       </c>
       <c r="H20" s="12" t="inlineStr">
@@ -2002,7 +1999,7 @@
       </c>
       <c r="G21" s="13" t="inlineStr">
         <is>
-          <t>C13 Design of System/Evidence/00 Common/C13.02 - SDLC Project List.xlsx</t>
+          <t>C13 Design of System/CDA/Process Map and Population/BSI.IT.23.C13.02 - SDLC Project List (population).xlsx</t>
         </is>
       </c>
       <c r="H21" s="12" t="inlineStr">
@@ -2044,7 +2041,7 @@
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>C13 Design of System/Evidence/S1 SecLending/C13.03 - SL DRA (Low).pdf</t>
+          <t>C13 Design of System/CPA/S1 Security Lending/BSI.IT.23.C13.03 - Security Lending Data Risk Assessment (Low).pdf</t>
         </is>
       </c>
       <c r="H22" s="12" t="inlineStr">
@@ -2086,7 +2083,7 @@
       </c>
       <c r="G23" s="13" t="inlineStr">
         <is>
-          <t>C13 Design of System/Evidence/S2 NDF/C13.04 - NDF DRA (High).pdf</t>
+          <t>C13 Design of System/CPA/S2 NDF/BSI.IT.23.C13.04 - NDF Data Risk Assessment (High).pdf</t>
         </is>
       </c>
       <c r="H23" s="12" t="inlineStr">
@@ -2128,7 +2125,7 @@
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
-          <t>C13 Design of System/Evidence/S1 SecLending/C13.05 - SL DRA approval and gates.docx</t>
+          <t>C13 Design of System/CPA/S1 Security Lending/BSI.IT.23.C13.05 - Security Lending DRA approval and gate history.docx</t>
         </is>
       </c>
       <c r="H24" s="12" t="inlineStr">
@@ -2170,7 +2167,7 @@
       </c>
       <c r="G25" s="13" t="inlineStr">
         <is>
-          <t>C13 Design of System/Evidence/S2 NDF/C13.06 - NDF DRA approval and gates.docx</t>
+          <t>C13 Design of System/CPA/S2 NDF/BSI.IT.23.C13.06 - NDF DRA approval and gate history.docx</t>
         </is>
       </c>
       <c r="H25" s="12" t="inlineStr">
@@ -2212,7 +2209,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>C13 Design of System/Evidence/S1 SecLending/C13.07 - SL EA approval 12-04-2025.msg</t>
+          <t>C13 Design of System/CPA/S1 Security Lending/BSI.IT.23.C13.07 - Security Lending EA approval 12-04-2025.msg</t>
         </is>
       </c>
       <c r="H26" s="12" t="inlineStr">
@@ -2254,7 +2251,7 @@
       </c>
       <c r="G27" s="13" t="inlineStr">
         <is>
-          <t>C13 Design of System/Evidence/S1 SecLending/C13.08 - SL EA Appian no impact 02-09-2026.msg</t>
+          <t>C13 Design of System/CPA/S1 Security Lending/BSI.IT.23.C13.08 - Security Lending EA Appian no impact 02-09-2026.msg</t>
         </is>
       </c>
       <c r="H27" s="12" t="inlineStr">
@@ -2296,7 +2293,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>C13 Design of System/Evidence/S1 SecLending/C13.09 - SL EA no ARB 05-12-2026.msg</t>
+          <t>C13 Design of System/CPA/S1 Security Lending/BSI.IT.23.C13.09 - Security Lending EA no ARB needed 05-12-2026.msg</t>
         </is>
       </c>
       <c r="H28" s="12" t="inlineStr">
@@ -2338,7 +2335,7 @@
       </c>
       <c r="G29" s="13" t="inlineStr">
         <is>
-          <t>C13 Design of System/Evidence/S2 NDF/C13.10 - NDF R01 EA sign-off 12-10-2025.msg</t>
+          <t>C13 Design of System/CPA/S2 NDF/BSI.IT.23.C13.10 - NDF R01 EA approval 12-10-2025.msg</t>
         </is>
       </c>
       <c r="H29" s="12" t="inlineStr">
@@ -2380,7 +2377,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>C13 Design of System/Evidence/S2 NDF/C13.11 - NDF R02 EA sign-off 03-24-2026.msg</t>
+          <t>C13 Design of System/CPA/S2 NDF/BSI.IT.23.C13.11 - NDF R02 EA approval 03-24-2026.msg</t>
         </is>
       </c>
       <c r="H30" s="12" t="inlineStr">
@@ -2422,7 +2419,7 @@
       </c>
       <c r="G31" s="13" t="inlineStr">
         <is>
-          <t>C25 Implement Deploy/Evidence/00 Common/C25.01 - 2026 SDLC process map.pdf</t>
+          <t>C25 Implement Deploy/CDA/Process Map and Population/BSI.IT.23.C25.01 - 2026 SDLC Process Map.pdf</t>
         </is>
       </c>
       <c r="H31" s="12" t="inlineStr">
@@ -2464,7 +2461,7 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>C25 Implement Deploy/Evidence/00 Common/C25.02 - SDLC Project List.xlsx</t>
+          <t>C25 Implement Deploy/CDA/Process Map and Population/BSI.IT.23.C25.02 - SDLC Project List (population).xlsx</t>
         </is>
       </c>
       <c r="H32" s="12" t="inlineStr">
@@ -2506,7 +2503,7 @@
       </c>
       <c r="G33" s="13" t="inlineStr">
         <is>
-          <t>C25 Implement Deploy/Evidence/S1 SecLending/C25.03 - SL R01 RLSE1271544 ticket.pdf</t>
+          <t>C25 Implement Deploy/CPA/S1 Security Lending/BSI.IT.23.C25.03 - Security Lending R01 ticket RLSE1271544.pdf</t>
         </is>
       </c>
       <c r="H33" s="12" t="inlineStr">
@@ -2548,7 +2545,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>C25 Implement Deploy/Evidence/S1 SecLending/C25.04 - SL R01 Deployment Plan.xlsx</t>
+          <t>C25 Implement Deploy/CPA/S1 Security Lending/BSI.IT.23.C25.04 - Security Lending R01 Deployment Plan.xlsx</t>
         </is>
       </c>
       <c r="H34" s="12" t="inlineStr">
@@ -2590,7 +2587,7 @@
       </c>
       <c r="G35" s="13" t="inlineStr">
         <is>
-          <t>C25 Implement Deploy/Evidence/S1 SecLending/C25.05 - SL R01 Functional doc.docx</t>
+          <t>C25 Implement Deploy/CPA/S1 Security Lending/BSI.IT.23.C25.05 - Security Lending R01 Functional doc.docx</t>
         </is>
       </c>
       <c r="H35" s="12" t="inlineStr">
@@ -2632,7 +2629,7 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>C25 Implement Deploy/Evidence/S1 SecLending/C25.06 - SL R02 RLSE1370716 ticket.pdf</t>
+          <t>C25 Implement Deploy/CPA/S1 Security Lending/BSI.IT.23.C25.06 - Security Lending R02 ticket RLSE1370716.pdf</t>
         </is>
       </c>
       <c r="H36" s="12" t="inlineStr">
@@ -2674,7 +2671,7 @@
       </c>
       <c r="G37" s="13" t="inlineStr">
         <is>
-          <t>C25 Implement Deploy/Evidence/S1 SecLending/C25.07 - SL R02 PIP.docx</t>
+          <t>C25 Implement Deploy/CPA/S1 Security Lending/BSI.IT.23.C25.07 - Security Lending R02 PIP.docx</t>
         </is>
       </c>
       <c r="H37" s="12" t="inlineStr">
@@ -2716,7 +2713,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>C25 Implement Deploy/Evidence/S2 NDF/C25.08 - NDF R01 RLSE1270306 ticket.pdf</t>
+          <t>C25 Implement Deploy/CPA/S2 NDF/BSI.IT.23.C25.08 - NDF R01 ticket RLSE1270306.pdf</t>
         </is>
       </c>
       <c r="H38" s="12" t="inlineStr">
@@ -2758,7 +2755,7 @@
       </c>
       <c r="G39" s="13" t="inlineStr">
         <is>
-          <t>C25 Implement Deploy/Evidence/S2 NDF/C25.09 - NDF R01 ticket screenshot.pdf</t>
+          <t>C25 Implement Deploy/CPA/S2 NDF/BSI.IT.23.C25.09 - NDF R01 ticket screenshot.pdf</t>
         </is>
       </c>
       <c r="H39" s="12" t="inlineStr">
@@ -2800,7 +2797,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>C25 Implement Deploy/Evidence/S2 NDF/C25.10 - NDF R01 PIP.docx</t>
+          <t>C25 Implement Deploy/CPA/S2 NDF/BSI.IT.23.C25.10 - NDF R01 PIP.docx</t>
         </is>
       </c>
       <c r="H40" s="12" t="inlineStr">
@@ -2842,7 +2839,7 @@
       </c>
       <c r="G41" s="13" t="inlineStr">
         <is>
-          <t>C25 Implement Deploy/Evidence/S2 NDF/C25.11 - NDF R02 RLSE1329424 ticket.pdf</t>
+          <t>C25 Implement Deploy/CPA/S2 NDF/BSI.IT.23.C25.11 - NDF R02 ticket RLSE1329424.pdf</t>
         </is>
       </c>
       <c r="H41" s="12" t="inlineStr">
@@ -2884,7 +2881,7 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>C25 Implement Deploy/Evidence/S2 NDF/C25.12 - NDF R02 ticket screenshot.pdf</t>
+          <t>C25 Implement Deploy/CPA/S2 NDF/BSI.IT.23.C25.12 - NDF R02 ticket screenshot.pdf</t>
         </is>
       </c>
       <c r="H42" s="12" t="inlineStr">
@@ -2926,7 +2923,7 @@
       </c>
       <c r="G43" s="13" t="inlineStr">
         <is>
-          <t>C25 Implement Deploy/Evidence/S2 NDF/C25.13 - NDF R02 PIP v1.3.docx</t>
+          <t>C25 Implement Deploy/CPA/S2 NDF/BSI.IT.23.C25.13 - NDF R02 PIP v1.3.docx</t>
         </is>
       </c>
       <c r="H43" s="12" t="inlineStr">
@@ -2968,7 +2965,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>C17 Solution Intent/Evidence/00 Common/C17.01 - 2025 SDLC process map.pdf</t>
+          <t>C17 Solution Intent/CDA/Process Map and Population/BSI.IT.23.C17.01 - 2025 SDLC Process Map (C17 listed).pdf</t>
         </is>
       </c>
       <c r="H44" s="12" t="inlineStr">
@@ -3010,7 +3007,7 @@
       </c>
       <c r="G45" s="13" t="inlineStr">
         <is>
-          <t>C17 Solution Intent/Evidence/00 Common/C17.02 - 2026 SDLC process map.pdf</t>
+          <t>C17 Solution Intent/CDA/Process Map and Population/BSI.IT.23.C17.02 - 2026 SDLC Process Map.pdf</t>
         </is>
       </c>
       <c r="H45" s="12" t="inlineStr">
@@ -3052,7 +3049,7 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>C17 Solution Intent/Evidence/00 Common/C17.03 - SDLC Project List.xlsx</t>
+          <t>C17 Solution Intent/CDA/Process Map and Population/BSI.IT.23.C17.03 - SDLC Project List (population).xlsx</t>
         </is>
       </c>
       <c r="H46" s="12" t="inlineStr">
@@ -3094,7 +3091,7 @@
       </c>
       <c r="G47" s="13" t="inlineStr">
         <is>
-          <t>C17 Solution Intent/Evidence/S1 SecLending/C17.04 - SL Single Design Feb 2026.pptx</t>
+          <t>C17 Solution Intent/CPA/S1 Security Lending/BSI.IT.23.C17.04 - Security Lending Single Design Feb 2026.pptx</t>
         </is>
       </c>
       <c r="H47" s="12" t="inlineStr">
@@ -3136,7 +3133,7 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>C17 Solution Intent/Evidence/S1 SecLending/C17.05 - SL EA approval 12-04-2025.msg</t>
+          <t>C17 Solution Intent/CPA/S1 Security Lending/BSI.IT.23.C17.05 - Security Lending EA approval 12-04-2025.msg</t>
         </is>
       </c>
       <c r="H48" s="12" t="inlineStr">
@@ -3178,7 +3175,7 @@
       </c>
       <c r="G49" s="13" t="inlineStr">
         <is>
-          <t>C17 Solution Intent/Evidence/S1 SecLending/C17.06 - SL EA Appian no impact 02-09-2026.msg</t>
+          <t>C17 Solution Intent/CPA/S1 Security Lending/BSI.IT.23.C17.06 - Security Lending EA Appian no impact 02-09-2026.msg</t>
         </is>
       </c>
       <c r="H49" s="12" t="inlineStr">
@@ -3220,7 +3217,7 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>C17 Solution Intent/Evidence/S1 SecLending/C17.07 - SL Single Design May 2026.pptx</t>
+          <t>C17 Solution Intent/CPA/S1 Security Lending/BSI.IT.23.C17.07 - Security Lending Single Design May 2026.pptx</t>
         </is>
       </c>
       <c r="H50" s="12" t="inlineStr">
@@ -3262,7 +3259,7 @@
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>C17 Solution Intent/Evidence/S1 SecLending/C17.08 - SL EA no ARB 05-12-2026.msg</t>
+          <t>C17 Solution Intent/CPA/S1 Security Lending/BSI.IT.23.C17.08 - Security Lending EA no ARB needed 05-12-2026.msg</t>
         </is>
       </c>
       <c r="H51" s="12" t="inlineStr">
@@ -3304,7 +3301,7 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>C17 Solution Intent/Evidence/S2 NDF/C17.09 - NDF R01 Technical Design.pptx</t>
+          <t>C17 Solution Intent/CPA/S2 NDF/BSI.IT.23.C17.09 - NDF R01 Single Technical Design.pptx</t>
         </is>
       </c>
       <c r="H52" s="12" t="inlineStr">
@@ -3346,7 +3343,7 @@
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>C17 Solution Intent/Evidence/S2 NDF/C17.10 - NDF R01 EA sign-off 12-10-2025.msg</t>
+          <t>C17 Solution Intent/CPA/S2 NDF/BSI.IT.23.C17.10 - NDF R01 EA approval 12-10-2025.msg</t>
         </is>
       </c>
       <c r="H53" s="12" t="inlineStr">
@@ -3388,7 +3385,7 @@
       </c>
       <c r="G54" s="13" t="inlineStr">
         <is>
-          <t>C17 Solution Intent/Evidence/S2 NDF/C17.11 - NDF R02 Technical Design.pptx</t>
+          <t>C17 Solution Intent/CPA/S2 NDF/BSI.IT.23.C17.11 - NDF R02 Single Technical Design.pptx</t>
         </is>
       </c>
       <c r="H54" s="12" t="inlineStr">
@@ -3430,7 +3427,7 @@
       </c>
       <c r="G55" s="13" t="inlineStr">
         <is>
-          <t>C17 Solution Intent/Evidence/S2 NDF/C17.12 - NDF R02 EA sign-off 03-24-2026.msg</t>
+          <t>C17 Solution Intent/CPA/S2 NDF/BSI.IT.23.C17.12 - NDF R02 EA approval 03-24-2026.msg</t>
         </is>
       </c>
       <c r="H55" s="12" t="inlineStr">
@@ -3472,7 +3469,7 @@
       </c>
       <c r="G56" s="13" t="inlineStr">
         <is>
-          <t>C17 Solution Intent/Evidence/S1 SecLending/C17.13 - SL gate dispositions.docx</t>
+          <t>C17 Solution Intent/CPA/S1 Security Lending/BSI.IT.23.C17.13 - Security Lending gate history.docx</t>
         </is>
       </c>
       <c r="H56" s="12" t="inlineStr">
@@ -3514,7 +3511,7 @@
       </c>
       <c r="G57" s="13" t="inlineStr">
         <is>
-          <t>C17 Solution Intent/Evidence/S2 NDF/C17.14 - NDF gate dispositions.docx</t>
+          <t>C17 Solution Intent/CPA/S2 NDF/BSI.IT.23.C17.14 - NDF gate history.docx</t>
         </is>
       </c>
       <c r="H57" s="12" t="inlineStr">
@@ -3556,7 +3553,7 @@
       </c>
       <c r="G58" s="13" t="inlineStr">
         <is>
-          <t>C4 Segregated Env/Evidence/00 Common/C4.01 - 2026 SDLC process map.pdf</t>
+          <t>C4 Segregated Env/CDA/Process Map and Population/BSI.IT.23.C4.01 - 2026 SDLC Process Map.pdf</t>
         </is>
       </c>
       <c r="H58" s="12" t="inlineStr">
@@ -3598,7 +3595,7 @@
       </c>
       <c r="G59" s="13" t="inlineStr">
         <is>
-          <t>C4 Segregated Env/Evidence/00 Common/C4.02 - SDLC Project List.xlsx</t>
+          <t>C4 Segregated Env/CDA/Process Map and Population/BSI.IT.23.C4.02 - SDLC Project List (population).xlsx</t>
         </is>
       </c>
       <c r="H59" s="12" t="inlineStr">
@@ -3640,7 +3637,7 @@
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>C4 Segregated Env/Evidence/S1 SecLending/C4.03 - SL Segregated Environments.docx</t>
+          <t>C4 Segregated Env/CPA/S1 Security Lending/BSI.IT.23.C4.03 - Security Lending Segregated Environments.docx</t>
         </is>
       </c>
       <c r="H60" s="12" t="inlineStr">
@@ -3682,7 +3679,7 @@
       </c>
       <c r="G61" s="13" t="inlineStr">
         <is>
-          <t>C4 Segregated Env/Evidence/S2 NDF/C4.04 - NDF R01 RLSE1270306 ticket.pdf</t>
+          <t>C4 Segregated Env/CPA/S2 NDF/BSI.IT.23.C4.04 - NDF R01 ticket RLSE1270306.pdf</t>
         </is>
       </c>
       <c r="H61" s="12" t="inlineStr">
@@ -3724,7 +3721,7 @@
       </c>
       <c r="G62" s="13" t="inlineStr">
         <is>
-          <t>C4 Segregated Env/Evidence/S2 NDF/C4.05 - NDF R02 RLSE1329424 ticket.pdf</t>
+          <t>C4 Segregated Env/CPA/S2 NDF/BSI.IT.23.C4.05 - NDF R02 ticket RLSE1329424.pdf</t>
         </is>
       </c>
       <c r="H62" s="12" t="inlineStr">
@@ -3766,7 +3763,7 @@
       </c>
       <c r="G63" s="13" t="inlineStr">
         <is>
-          <t>C4 Segregated Env/Evidence/S1 SecLending/C4.06 - SL R01 RLSE1271544 ticket.pdf</t>
+          <t>C4 Segregated Env/CPA/S1 Security Lending/BSI.IT.23.C4.06 - Security Lending R01 ticket RLSE1271544.pdf</t>
         </is>
       </c>
       <c r="H63" s="12" t="inlineStr">
@@ -3808,7 +3805,7 @@
       </c>
       <c r="G64" s="13" t="inlineStr">
         <is>
-          <t>C4 Segregated Env/Evidence/S1 SecLending/C4.07 - SL R02 RLSE1370716 ticket.pdf</t>
+          <t>C4 Segregated Env/CPA/S1 Security Lending/BSI.IT.23.C4.07 - Security Lending R02 ticket RLSE1370716.pdf</t>
         </is>
       </c>
       <c r="H64" s="12" t="inlineStr">
@@ -3850,7 +3847,7 @@
       </c>
       <c r="G65" s="13" t="inlineStr">
         <is>
-          <t>C4 Segregated Env/Evidence/S2 NDF/C4.08 - NDF Segregated Environments.docx</t>
+          <t>C4 Segregated Env/CPA/S2 NDF/BSI.IT.23.C4.08 - NDF Segregated Environments.docx</t>
         </is>
       </c>
       <c r="H65" s="12" t="inlineStr">
@@ -3970,7 +3967,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>

</xml_diff>